<commit_message>
Add MVP country data pipeline API and tests
</commit_message>
<xml_diff>
--- a/data/sample/05_prototype_dataset.xlsx
+++ b/data/sample/05_prototype_dataset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\X1\EduPath\data\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A93EAA0-17CB-45DC-9E9A-96A4FB790679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF80358-4939-4ECF-A7D2-395F9E10710C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="9600" windowHeight="10200" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="countries" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="74">
   <si>
     <t>university_id</t>
   </si>
@@ -181,6 +181,75 @@
   </si>
   <si>
     <t>https://www.i.u-tokyo.ac.jp/ist_en/en-course/prg.shtml</t>
+  </si>
+  <si>
+    <t>country_name</t>
+  </si>
+  <si>
+    <t>region</t>
+  </si>
+  <si>
+    <t>capital_city</t>
+  </si>
+  <si>
+    <t>currency_code</t>
+  </si>
+  <si>
+    <t>main_language</t>
+  </si>
+  <si>
+    <t>estimated_living_cost</t>
+  </si>
+  <si>
+    <t>cost_currency</t>
+  </si>
+  <si>
+    <t>Japan</t>
+  </si>
+  <si>
+    <t>East Asia</t>
+  </si>
+  <si>
+    <t>Japanese</t>
+  </si>
+  <si>
+    <t>https://www.studyinjapan.go.jp/en/</t>
+  </si>
+  <si>
+    <t>country_sg</t>
+  </si>
+  <si>
+    <t>Singapore</t>
+  </si>
+  <si>
+    <t>Southeast Asia</t>
+  </si>
+  <si>
+    <t>SGD</t>
+  </si>
+  <si>
+    <t>English, Malay, Mandarin, Tamil</t>
+  </si>
+  <si>
+    <t>https://www.moe.gov.sg/</t>
+  </si>
+  <si>
+    <t>country_my</t>
+  </si>
+  <si>
+    <t>Malaysia</t>
+  </si>
+  <si>
+    <t>Kuala Lumpur</t>
+  </si>
+  <si>
+    <t>MYR</t>
+  </si>
+  <si>
+    <t>Malay</t>
+  </si>
+  <si>
+    <t>https://www.mqa.gov.my/</t>
   </si>
 </sst>
 </file>
@@ -236,7 +305,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -254,6 +323,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -535,12 +613,151 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" customWidth="1"/>
+    <col min="1" max="1" width="10.7265625" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.08984375" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.26953125" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.08984375" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.90625" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.36328125" style="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28.54296875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="10.81640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.7265625" style="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.7265625" style="10"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J2" s="11">
+        <v>46236</v>
+      </c>
+      <c r="K2" s="11">
+        <v>46236</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="J3" s="11">
+        <v>46236</v>
+      </c>
+      <c r="K3" s="11">
+        <v>46236</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J4" s="11">
+        <v>46236</v>
+      </c>
+      <c r="K4" s="11">
+        <v>46236</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{4B37C802-BCE8-47E9-9188-AEDAE3B60B80}"/>
+    <hyperlink ref="I3" r:id="rId2" xr:uid="{B832C158-4650-4118-91DB-08F899FC69EE}"/>
+    <hyperlink ref="I4" r:id="rId3" xr:uid="{BFB7E0CB-AE2C-48E4-BD05-E2FDAD9CA8F1}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add MVP scholarship data pipeline API and tests
</commit_message>
<xml_diff>
--- a/data/sample/05_prototype_dataset.xlsx
+++ b/data/sample/05_prototype_dataset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\X1\EduPath\data\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF80358-4939-4ECF-A7D2-395F9E10710C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C3232CA-9355-4B3D-A09D-E57BA9FA640A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="countries" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="108">
   <si>
     <t>university_id</t>
   </si>
@@ -250,6 +250,108 @@
   </si>
   <si>
     <t>https://www.mqa.gov.my/</t>
+  </si>
+  <si>
+    <t>scholarship_id</t>
+  </si>
+  <si>
+    <t>scholarship_name</t>
+  </si>
+  <si>
+    <t>provider_name</t>
+  </si>
+  <si>
+    <t>provider_type</t>
+  </si>
+  <si>
+    <t>host_university_id</t>
+  </si>
+  <si>
+    <t>eligible_nationalities</t>
+  </si>
+  <si>
+    <t>fields_of_study</t>
+  </si>
+  <si>
+    <t>age_limit</t>
+  </si>
+  <si>
+    <t>funding_type</t>
+  </si>
+  <si>
+    <t>tuition_coverage</t>
+  </si>
+  <si>
+    <t>monthly_allowance</t>
+  </si>
+  <si>
+    <t>allowance_currency</t>
+  </si>
+  <si>
+    <t>travel_allowance</t>
+  </si>
+  <si>
+    <t>accommodation_support</t>
+  </si>
+  <si>
+    <t>health_insurance</t>
+  </si>
+  <si>
+    <t>required_documents</t>
+  </si>
+  <si>
+    <t>application_opening_date</t>
+  </si>
+  <si>
+    <t>scholarship_status</t>
+  </si>
+  <si>
+    <t>application_cycle</t>
+  </si>
+  <si>
+    <t>data_quality_status</t>
+  </si>
+  <si>
+    <t>sch_jp_001</t>
+  </si>
+  <si>
+    <t>Japanese Government (MEXT) Scholarship - University Recommendation (General Selection), IST, October 2027</t>
+  </si>
+  <si>
+    <t>Ministry of Education, Culture, Sports, Science and Technology (MEXT)</t>
+  </si>
+  <si>
+    <t>Government</t>
+  </si>
+  <si>
+    <t>Master, PhD</t>
+  </si>
+  <si>
+    <t>Computer Science, Mathematical Informatics, Information Physics and Computing, Information and Communication Engineering, Mechano-Informatics, Creative Informatics</t>
+  </si>
+  <si>
+    <t>Fully Funded</t>
+  </si>
+  <si>
+    <t>Exam fee, entrance fee, and tuition exempted</t>
+  </si>
+  <si>
+    <t>Round-trip travel expenses under specified conditions</t>
+  </si>
+  <si>
+    <t>Application form, academic transcripts, GPA calculation form, graduation or degree certificate, English proficiency certificate, research summary, research achievements if applicable, field of study and research plan, recommendation letter, passport copy, conditional acceptance of prospective supervisor, examination fee receipt</t>
+  </si>
+  <si>
+    <t>upcoming</t>
+  </si>
+  <si>
+    <t>https://www.i.u-tokyo.ac.jp/edu/inter_ex/oir/scholarship_e.shtml</t>
+  </si>
+  <si>
+    <t>https://www.i.u-tokyo.ac.jp/edu/MEXT_General_Guidelines_E_Oct2027.pdf</t>
+  </si>
+  <si>
+    <t>verified</t>
   </si>
 </sst>
 </file>
@@ -305,7 +407,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -331,6 +433,12 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1033,9 +1141,225 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A67CBE2-A81D-49C2-BA44-C4091CD9D487}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="14.08984375" style="12" customWidth="1"/>
+    <col min="2" max="2" width="23.453125" style="12" customWidth="1"/>
+    <col min="3" max="3" width="29.08984375" style="12" customWidth="1"/>
+    <col min="4" max="4" width="22.36328125" style="12" customWidth="1"/>
+    <col min="5" max="5" width="18.26953125" style="12" customWidth="1"/>
+    <col min="6" max="6" width="19.54296875" style="12" customWidth="1"/>
+    <col min="7" max="7" width="19.36328125" style="12" customWidth="1"/>
+    <col min="8" max="8" width="13.90625" style="12" customWidth="1"/>
+    <col min="9" max="9" width="27.90625" style="12" customWidth="1"/>
+    <col min="10" max="10" width="19.54296875" style="12" customWidth="1"/>
+    <col min="11" max="11" width="12.54296875" style="12" customWidth="1"/>
+    <col min="12" max="12" width="16.26953125" style="12" customWidth="1"/>
+    <col min="13" max="14" width="12.54296875" style="12" customWidth="1"/>
+    <col min="15" max="15" width="14.1796875" style="12" customWidth="1"/>
+    <col min="16" max="16" width="14.81640625" style="12" customWidth="1"/>
+    <col min="17" max="17" width="19.08984375" style="12" customWidth="1"/>
+    <col min="18" max="18" width="21.81640625" style="12" customWidth="1"/>
+    <col min="19" max="19" width="14.36328125" style="12" customWidth="1"/>
+    <col min="20" max="20" width="17.36328125" style="12" customWidth="1"/>
+    <col min="21" max="21" width="15.26953125" style="12" customWidth="1"/>
+    <col min="22" max="22" width="30.453125" style="12" customWidth="1"/>
+    <col min="23" max="23" width="24.08984375" style="12" customWidth="1"/>
+    <col min="24" max="24" width="22.7265625" style="12" customWidth="1"/>
+    <col min="25" max="25" width="8.7265625" style="12"/>
+    <col min="26" max="26" width="17.26953125" style="12" customWidth="1"/>
+    <col min="27" max="27" width="21" style="12" customWidth="1"/>
+    <col min="28" max="28" width="26.90625" style="12" customWidth="1"/>
+    <col min="29" max="29" width="17.7265625" style="12" customWidth="1"/>
+    <col min="30" max="30" width="19.36328125" style="12" customWidth="1"/>
+    <col min="31" max="31" width="23.08984375" style="12" customWidth="1"/>
+    <col min="32" max="32" width="16.6328125" style="12" customWidth="1"/>
+    <col min="33" max="16384" width="8.7265625" style="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:32" s="13" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="T1" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="U1" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V1" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="W1" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="X1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y1" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="Z1" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="AA1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="AB1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="AC1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="AD1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="AE1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF1" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:32" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>143000</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="W2" s="3">
+        <v>46314</v>
+      </c>
+      <c r="X2" s="3">
+        <v>46325</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="Z2" s="1">
+        <v>2027</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="AC2" s="3">
+        <v>46236</v>
+      </c>
+      <c r="AD2" s="3">
+        <v>46236</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add MVP program recommendation engine API and tests
</commit_message>
<xml_diff>
--- a/data/sample/05_prototype_dataset.xlsx
+++ b/data/sample/05_prototype_dataset.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\X1\EduPath\data\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C3232CA-9355-4B3D-A09D-E57BA9FA640A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AB33E70-424C-4ED3-83EA-54BAE5F8030A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="countries" sheetId="1" r:id="rId1"/>
     <sheet name="universities" sheetId="2" r:id="rId2"/>
     <sheet name="programs" sheetId="3" r:id="rId3"/>
     <sheet name="scholarships" sheetId="4" r:id="rId4"/>
+    <sheet name="user_profiles" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="130">
   <si>
     <t>university_id</t>
   </si>
@@ -352,6 +353,72 @@
   </si>
   <si>
     <t>verified</t>
+  </si>
+  <si>
+    <t>user_id</t>
+  </si>
+  <si>
+    <t>nationality</t>
+  </si>
+  <si>
+    <t>current_education_level</t>
+  </si>
+  <si>
+    <t>target_degree_level</t>
+  </si>
+  <si>
+    <t>preferred_major</t>
+  </si>
+  <si>
+    <t>gpa</t>
+  </si>
+  <si>
+    <t>ielts_score</t>
+  </si>
+  <si>
+    <t>toefl_score</t>
+  </si>
+  <si>
+    <t>annual_budget</t>
+  </si>
+  <si>
+    <t>budget_currency</t>
+  </si>
+  <si>
+    <t>preferred_countries</t>
+  </si>
+  <si>
+    <t>scholarship_required</t>
+  </si>
+  <si>
+    <t>preferred_funding_type</t>
+  </si>
+  <si>
+    <t>preferred_intake</t>
+  </si>
+  <si>
+    <t>saved_universities</t>
+  </si>
+  <si>
+    <t>saved_scholarships</t>
+  </si>
+  <si>
+    <t>recommendation_history</t>
+  </si>
+  <si>
+    <t>user_test_001</t>
+  </si>
+  <si>
+    <t>Myanmar</t>
+  </si>
+  <si>
+    <t>Bachelor</t>
+  </si>
+  <si>
+    <t>Computer Science</t>
+  </si>
+  <si>
+    <t>October</t>
   </si>
 </sst>
 </file>
@@ -1362,4 +1429,134 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59C51B4D-AB24-43CB-AC94-6851E32FE473}">
+  <dimension ref="A1:R2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.6328125" customWidth="1"/>
+    <col min="7" max="7" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.08984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="N1" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q1" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" t="s">
+        <v>128</v>
+      </c>
+      <c r="F2">
+        <v>3.5</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>6.5</v>
+      </c>
+      <c r="J2">
+        <v>600000</v>
+      </c>
+      <c r="K2" t="s">
+        <v>47</v>
+      </c>
+      <c r="L2" t="s">
+        <v>58</v>
+      </c>
+      <c r="M2" t="b">
+        <v>1</v>
+      </c>
+      <c r="N2" t="s">
+        <v>100</v>
+      </c>
+      <c r="O2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>